<commit_message>
removed present bugs apis working as it should be
</commit_message>
<xml_diff>
--- a/backend/excel/work_order.xlsx
+++ b/backend/excel/work_order.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="4Dome" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="3Dome" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Input" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="3Dome" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -312,34 +313,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -485,7 +486,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="4"/>
@@ -700,8 +701,52 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="D1:D6"/>
+  <sheetFormatPr defaultColWidth="8.5625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D1" s="1" t="n">
+        <v>2353</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D2" s="1" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D3" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D4" s="1" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D6" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="4"/>
@@ -713,11 +758,11 @@
         <v>0</v>
       </c>
       <c r="D1" s="3" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="E1" s="4" t="n">
         <f aca="false">(D1-2*D3)/3</f>
-        <v>0</v>
+        <v>28.3333333333333</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -725,11 +770,10 @@
         <v>1</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="E2" s="4" t="n">
-        <f aca="false">D3</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -737,11 +781,10 @@
         <v>2</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E3" s="4" t="n">
-        <f aca="false">D3/2</f>
-        <v>0</v>
+        <v>5263</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -749,11 +792,10 @@
         <v>3</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="E4" s="4" t="n">
-        <f aca="false">(D1-2*D3)/2</f>
-        <v>0</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -762,8 +804,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="4" t="n">
-        <f aca="false">D3</f>
-        <v>0</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -771,17 +812,17 @@
         <v>4</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="E6" s="4" t="n">
         <f aca="false">D3</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E7" s="4" t="n">
         <f aca="false">D2-2*D3</f>
-        <v>0</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -790,7 +831,7 @@
       </c>
       <c r="E8" s="4" t="n">
         <f aca="false">D3/2</f>
-        <v>0</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -799,7 +840,7 @@
       </c>
       <c r="E9" s="4" t="n">
         <f aca="false">D3/4</f>
-        <v>0</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -808,7 +849,7 @@
       </c>
       <c r="E10" s="4" t="n">
         <f aca="false">D2</f>
-        <v>0</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -817,7 +858,7 @@
       </c>
       <c r="E11" s="4" t="n">
         <f aca="false">D2</f>
-        <v>0</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -825,8 +866,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="4" t="n">
-        <f aca="false">D3/3.5</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -835,7 +875,7 @@
       </c>
       <c r="E13" s="4" t="n">
         <f aca="false">D4*0.22</f>
-        <v>0</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -844,7 +884,7 @@
       </c>
       <c r="E14" s="4" t="n">
         <f aca="false">D1-2*D3</f>
-        <v>0</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -852,8 +892,7 @@
         <v>12</v>
       </c>
       <c r="E15" s="4" t="n">
-        <f aca="false">D4+D3</f>
-        <v>0</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -862,7 +901,7 @@
       </c>
       <c r="E16" s="4" t="n">
         <f aca="false">D2</f>
-        <v>0</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
last update till we keep excel as the calculation engine before switching to spreadsheets
</commit_message>
<xml_diff>
--- a/backend/excel/work_order.xlsx
+++ b/backend/excel/work_order.xlsx
@@ -758,11 +758,11 @@
         <v>0</v>
       </c>
       <c r="D1" s="3" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="E1" s="4" t="n">
         <f aca="false">(D1-2*D3)/3</f>
-        <v>28.3333333333333</v>
+        <v>-20.6666666666667</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -770,7 +770,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="E2" s="4" t="n">
         <v>5</v>
@@ -781,7 +781,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>7</v>
+        <v>75</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>5263</v>
@@ -792,7 +792,7 @@
         <v>3</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>55</v>
+        <v>3</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>52</v>
@@ -812,17 +812,17 @@
         <v>4</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="E6" s="4" t="n">
         <f aca="false">D3</f>
-        <v>7</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E7" s="4" t="n">
         <f aca="false">D2-2*D3</f>
-        <v>64</v>
+        <v>-62</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -831,7 +831,7 @@
       </c>
       <c r="E8" s="4" t="n">
         <f aca="false">D3/2</f>
-        <v>3.5</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -840,7 +840,7 @@
       </c>
       <c r="E9" s="4" t="n">
         <f aca="false">D3/4</f>
-        <v>1.75</v>
+        <v>18.75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -849,7 +849,7 @@
       </c>
       <c r="E10" s="4" t="n">
         <f aca="false">D2</f>
-        <v>78</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -858,7 +858,7 @@
       </c>
       <c r="E11" s="4" t="n">
         <f aca="false">D2</f>
-        <v>78</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -875,7 +875,7 @@
       </c>
       <c r="E13" s="4" t="n">
         <f aca="false">D4*0.22</f>
-        <v>12.1</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -884,7 +884,7 @@
       </c>
       <c r="E14" s="4" t="n">
         <f aca="false">D1-2*D3</f>
-        <v>85</v>
+        <v>-62</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -901,7 +901,7 @@
       </c>
       <c r="E16" s="4" t="n">
         <f aca="false">D2</f>
-        <v>78</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>